<commit_message>
Built new resumes in tabular format
</commit_message>
<xml_diff>
--- a/peopleLikeMe/data/dam_resume.xlsx
+++ b/peopleLikeMe/data/dam_resume.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DeloresMincarelli\Documents\Portfolio\peopleLikeMe\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{74B5D018-9DC9-4C2C-AB42-1755631A9826}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{096104C1-786F-4BA6-8DD7-B49851AA09F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{CEA2BB9E-CFA2-49BB-8AD4-3B83B24091B6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="43">
   <si>
     <t>ResumeID</t>
   </si>
@@ -121,6 +121,60 @@
   </si>
   <si>
     <t>Automated calculation of Sensitivity, Specificity, Accuracy and Confidence Intervals for clinical study results.</t>
+  </si>
+  <si>
+    <t>Data Scientist</t>
+  </si>
+  <si>
+    <t>Provided significance tests for cardiac surgery department (a) to determine volumes did not support reduction of
+staff (b) comparing operational efficiencies leading to shared learning between departments</t>
+  </si>
+  <si>
+    <t>Architected, programmed &amp; delivered seminal work-flow to calculate utilization of anesthesiologists site wide.</t>
+  </si>
+  <si>
+    <t>Provided data &amp; dashboard to influence decision to use median procedure time vs "one size fits all" for high volume
+procedures in cardiac surgery department.</t>
+  </si>
+  <si>
+    <t>Created views, stored procedures and tables underpinning nurse scheduling optimization project; architected process
+needed to ETL historical data and do daily refreshes of the data.</t>
+  </si>
+  <si>
+    <t>Prototyped optimization of nurse shift preferences with daily demand</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>BS Chemical Engineering</t>
+  </si>
+  <si>
+    <t>MS Business Analytics</t>
+  </si>
+  <si>
+    <t>Skills</t>
+  </si>
+  <si>
+    <t>Critical Thinking</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>Problem Solving</t>
+  </si>
+  <si>
+    <t>Analysis</t>
+  </si>
+  <si>
+    <t>PowerBI</t>
+  </si>
+  <si>
+    <t>Tableau</t>
   </si>
 </sst>
 </file>
@@ -495,12 +549,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{214867AD-8B1C-4F22-9FB7-BAE050E647DB}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="3" width="24.6640625" customWidth="1"/>
     <col min="5" max="5" width="64.77734375" customWidth="1"/>
-    <col min="7" max="7" width="18.109375" customWidth="1"/>
+    <col min="6" max="7" width="18.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -560,7 +614,7 @@
         <v>9</v>
       </c>
       <c r="F3">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -570,6 +624,9 @@
       <c r="A4">
         <v>1</v>
       </c>
+      <c r="B4" t="s">
+        <v>6</v>
+      </c>
       <c r="C4" t="s">
         <v>17</v>
       </c>
@@ -580,7 +637,7 @@
         <v>10</v>
       </c>
       <c r="F4">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -590,6 +647,9 @@
       <c r="A5">
         <v>1</v>
       </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
       <c r="C5" t="s">
         <v>17</v>
       </c>
@@ -600,7 +660,7 @@
         <v>11</v>
       </c>
       <c r="F5">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -610,6 +670,9 @@
       <c r="A6">
         <v>1</v>
       </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
       <c r="C6" t="s">
         <v>17</v>
       </c>
@@ -620,7 +683,7 @@
         <v>12</v>
       </c>
       <c r="F6">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -630,6 +693,9 @@
       <c r="A7">
         <v>1</v>
       </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
       <c r="C7" t="s">
         <v>17</v>
       </c>
@@ -640,7 +706,7 @@
         <v>13</v>
       </c>
       <c r="F7">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -650,6 +716,9 @@
       <c r="A8">
         <v>1</v>
       </c>
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
       <c r="C8" t="s">
         <v>16</v>
       </c>
@@ -660,7 +729,7 @@
         <v>14</v>
       </c>
       <c r="F8">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -670,6 +739,9 @@
       <c r="A9">
         <v>1</v>
       </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
       <c r="C9" t="s">
         <v>19</v>
       </c>
@@ -683,13 +755,16 @@
         <v>12</v>
       </c>
       <c r="G9">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>1</v>
       </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
       <c r="C10" t="s">
         <v>19</v>
       </c>
@@ -703,13 +778,16 @@
         <v>12</v>
       </c>
       <c r="G10">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>1</v>
       </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
       <c r="C11" t="s">
         <v>19</v>
       </c>
@@ -723,13 +801,16 @@
         <v>12</v>
       </c>
       <c r="G11">
-        <v>48</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>1</v>
       </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
       <c r="C12" t="s">
         <v>23</v>
       </c>
@@ -743,13 +824,16 @@
         <v>4</v>
       </c>
       <c r="G12">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1</v>
       </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
       <c r="C13" t="s">
         <v>23</v>
       </c>
@@ -763,13 +847,16 @@
         <v>4</v>
       </c>
       <c r="G13">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>1</v>
       </c>
+      <c r="B14" t="s">
+        <v>6</v>
+      </c>
       <c r="C14" t="s">
         <v>23</v>
       </c>
@@ -783,72 +870,254 @@
         <v>4</v>
       </c>
       <c r="G14">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15">
+        <v>14</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F15">
+        <v>36</v>
+      </c>
+      <c r="G15">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16">
+        <v>15</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16">
+        <v>36</v>
+      </c>
+      <c r="G16">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17">
+        <v>16</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17">
+        <v>36</v>
+      </c>
+      <c r="G17">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18">
+        <v>17</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18">
+        <v>36</v>
+      </c>
+      <c r="G18">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19">
+        <v>18</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F19">
+        <v>36</v>
+      </c>
+      <c r="G19">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20">
+        <v>19</v>
+      </c>
+      <c r="E20" t="s">
+        <v>34</v>
+      </c>
+      <c r="G20">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>32</v>
+      </c>
+      <c r="D21">
+        <v>20</v>
+      </c>
+      <c r="E21" t="s">
+        <v>33</v>
+      </c>
+      <c r="G21">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22">
+        <v>21</v>
+      </c>
+      <c r="E22" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23">
+        <v>22</v>
+      </c>
+      <c r="E23" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24">
+        <v>23</v>
+      </c>
+      <c r="E24" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25">
+        <v>24</v>
+      </c>
+      <c r="E25" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26">
+        <v>25</v>
+      </c>
+      <c r="E26" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>1</v>
+      </c>
+      <c r="B27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27">
+        <v>26</v>
+      </c>
+      <c r="E27" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>1</v>
+      </c>
+      <c r="B28" t="s">
+        <v>35</v>
+      </c>
+      <c r="D28">
+        <v>27</v>
+      </c>
+      <c r="E28" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>